<commit_message>
Arbitrum sweep: CEH $318k payroll hub folded in, register + workbook updated, Arbitrum FY25 tab added
</commit_message>
<xml_diff>
--- a/ZeroX_wallet_register_LOCKED.xlsx
+++ b/ZeroX_wallet_register_LOCKED.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Register" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buckets" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investor Reconciliation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arbitrum FY25" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +49,11 @@
       <sz val="9"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="00B26B00"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
     <font>
@@ -55,6 +61,14 @@
     </font>
     <font>
       <color rgb="00B26B00"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3A2E"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="8">
@@ -121,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,16 +167,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -528,16 +548,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -550,7 +570,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-06 from on-chain trace · period to 31 Dec 2025 · 99.79% identified</t>
+          <t>Generated 2026-06-11 · Ethereum + Base + Arbitrum · period to 31 Dec 2025 · see Arbitrum FY25 tab for cross-chain payroll</t>
         </is>
       </c>
     </row>
@@ -577,12 +597,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>In $</t>
+          <t>In $ (eth+base)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Out $</t>
+          <t>Out $ (eth+base)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -1404,7 +1424,7 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>Dev/supplier.</t>
+          <t>Dev/payroll hub. Group paid $378k total: $318k on Arbitrum (monthly payroll Feb-Sep 2025 from W3/W4) + $60k mainnet (Oct-Dec 2025). CEH distributed on Arbitrum to team/contractors. Invoice 011 (to ST0x BVI) papers the Dec mainnet leg. Material FY25 expense not in eth+base map - flag Tom Fleming.</t>
         </is>
       </c>
     </row>
@@ -2934,22 +2954,22 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>0x4e5bd3cf829010280f76754b49921d4e1448b8cf</t>
+          <t>0x1d56a5ed5cbeaa8885bb61c820b7f897da00531c</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>Safe (Base)</t>
+          <t>Dave Meister (personal)</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Treasury / liquidity (excluded from accounting)</t>
-        </is>
-      </c>
-      <c r="D77" s="11" t="inlineStr">
-        <is>
-          <t>Treasury / liquidity (excluded)</t>
+          <t>Team / contractor</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>Counterparty (registered)</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
@@ -2960,38 +2980,137 @@
       </c>
       <c r="G77" s="8" t="inlineStr">
         <is>
-          <t>Group wallet.</t>
+          <t>CEH Arbitrum payee, ~$36k Mar-May 2025. NOT an alias of the CEH wallet (verified on-chain). Personal DeFi (Morpho/Raindex).</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
+          <t>0x1f7bc4da1a0c2e49d7ef542f74cd46a3fe592cb1</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Kraken deposit (Arbitrum)</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Own rails</t>
+        </is>
+      </c>
+      <c r="D78" s="10" t="inlineStr">
+        <is>
+          <t>Own rails / DeFi infra (excluded)</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="8" t="inlineStr">
+        <is>
+          <t>Arbitrum off-ramp deposit address, ~$42k 2025. Own rails, excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>0x4e5bd3cf829010280f76754b49921d4e1448b8cf</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Safe (Base)</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Treasury / liquidity (excluded from accounting)</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>Treasury / liquidity (excluded)</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="8" t="inlineStr">
+        <is>
+          <t>Group wallet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>0xdf1802c9ab5ed41615cc8db10ee8c1c0ea56dbc7</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>David Atkinson (Rain wallet)</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Team / contractor</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>Counterparty (registered)</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="8" t="inlineStr">
+        <is>
+          <t>CEH Arbitrum payee, ~$27k Feb-Sep 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
           <t>0xe70d821f3462a074e63b42d0aac6523faae1d611</t>
         </is>
       </c>
-      <c r="B78" s="5" t="inlineStr">
+      <c r="B81" s="5" t="inlineStr">
         <is>
           <t>Safe — issuance (wtSPYM / wtMSTR)</t>
         </is>
       </c>
-      <c r="C78" s="5" t="inlineStr">
+      <c r="C81" s="5" t="inlineStr">
         <is>
           <t>Treasury / liquidity (excluded from accounting)</t>
         </is>
       </c>
-      <c r="D78" s="11" t="inlineStr">
+      <c r="D81" s="11" t="inlineStr">
         <is>
           <t>Treasury / liquidity (excluded)</t>
         </is>
       </c>
-      <c r="E78" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F78" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G78" s="8" t="inlineStr">
+      <c r="E81" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" s="8" t="inlineStr">
         <is>
           <t>Token issuance. S01 intercompany.</t>
         </is>
@@ -3008,136 +3127,113 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Accounting buckets (USD, stablecoin movements)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+          <t>Accounting buckets (USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Figures below are Ethereum + Base. Arbitrum FY25 payroll ($318k via CEH) is on the Arbitrum FY25 tab; 2026 Arbitrum trading (~$29m) is post-period FY26 and excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Internal / own (operating)</t>
         </is>
       </c>
-      <c r="B4" s="14" t="n">
+      <c r="B5" s="16" t="n">
         <v>3468957</v>
       </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>Own wallets, excluded from counterparty analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Registered counterparties</t>
         </is>
       </c>
-      <c r="B5" s="14" t="n">
+      <c r="B6" s="16" t="n">
         <v>2142634</v>
       </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>Named investors + counterparties</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Own rails (exchange/bridge/DeFi)</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="n">
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Own rails (exch/bridge/DeFi)</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
         <v>1075648</v>
       </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>Kraken, Gemini, LI.FI, Uniswap, Aave etc — excluded</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Treasury / liquidity</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B8" s="16" t="n">
         <v>516666</v>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>Safes, BitGo — excluded from accounting</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>Unregistered (sub-threshold dust)</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>15175</v>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>Tiny addresses below display cutoff — immaterial</t>
-        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>TOTAL classified</t>
+          <t>Unregistered (sub-threshold dust)</t>
         </is>
       </c>
       <c r="B9" s="16" t="n">
+        <v>15175</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL classified (eth+base)</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="n">
         <v>7219080</v>
       </c>
-      <c r="C9" s="15" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>IDENTIFIED</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="n">
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>IDENTIFIED (eth+base)</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="n">
         <v>7203905</v>
       </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>99.79% of all on-chain movement</t>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Identified = 99.79% of eth+base movement</t>
         </is>
       </c>
     </row>
@@ -3159,20 +3255,13 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="66" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Investor reconciliation — on-chain vs booked (Count 951) vs your master list</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>USD. 'Your list' is in-period unless noted. Blank = not present in that source.</t>
+          <t>Investor reconciliation — on-chain vs booked (951) vs your list</t>
         </is>
       </c>
     </row>
@@ -3218,7 +3307,7 @@
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Booked + on-chain; deliberately off your list</t>
+          <t>Booked + on-chain; off your list by design</t>
         </is>
       </c>
     </row>
@@ -3239,7 +3328,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Reconciles in aggregate; Dec tranche dates/legs differ — align with Count</t>
+          <t>Reconciles in aggregate; Dec tranche dates differ</t>
         </is>
       </c>
     </row>
@@ -3260,7 +3349,7 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>$200k ASA tied; Dec $100k SAFT mostly post-period/unfunded (~$76k); +$24k on-chain over booked</t>
+          <t>$200k ASA tied; Dec $100k SAFT mostly post-period</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3368,7 @@
       <c r="D8" s="7" t="n">
         <v>100000</v>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -3300,7 +3389,7 @@
       <c r="D9" s="7" t="n">
         <v>70000</v>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -3323,7 +3412,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Cash matches; the $90k combined + $25k commission are non-cash (warrant/ASA)</t>
+          <t>Cash matches; $90k+$25k are non-cash</t>
         </is>
       </c>
     </row>
@@ -3342,7 +3431,7 @@
       <c r="D11" s="7" t="n">
         <v>25000</v>
       </c>
-      <c r="E11" s="17" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -3363,9 +3452,9 @@
       <c r="D12" s="7" t="n">
         <v>10000</v>
       </c>
-      <c r="E12" s="17" t="inlineStr">
-        <is>
-          <t>MATCH (routed via Kraken)</t>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3473,7 @@
       <c r="D13" s="7" t="n">
         <v>10000</v>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E13" s="19" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -3405,7 +3494,7 @@
       <c r="D14" s="7" t="n">
         <v>2400</v>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="E14" s="19" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -3422,16 +3511,16 @@
       <c r="D15" s="7" t="n">
         <v>33000</v>
       </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>FIAT to bank — reconcile vs Revolut, confirm booked</t>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>FIAT to bank — reconcile vs Revolut</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Vantage Alpha LLC (Nick Thompson)</t>
+          <t>Vantage Alpha LLC</t>
         </is>
       </c>
       <c r="B16" s="5" t="n"/>
@@ -3439,16 +3528,16 @@
       <c r="D16" s="7" t="n">
         <v>30000</v>
       </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>FIAT, email-only, no agreement ref — verify</t>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>FIAT, email-only — verify</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>CTRL-H Ltd (Laurent Schonbach)</t>
+          <t>CTRL-H Ltd</t>
         </is>
       </c>
       <c r="B17" s="5" t="n"/>
@@ -3456,9 +3545,9 @@
       <c r="D17" s="7" t="n">
         <v>15000</v>
       </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>FIAT to bank — confirm received &amp; booked</t>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>FIAT to bank</t>
         </is>
       </c>
     </row>
@@ -3473,9 +3562,9 @@
       <c r="D18" s="7" t="n">
         <v>12500</v>
       </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>FIAT to bank — confirm received &amp; booked</t>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>FIAT to bank</t>
         </is>
       </c>
     </row>
@@ -3490,9 +3579,9 @@
       <c r="D19" s="7" t="n">
         <v>11750</v>
       </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>FIAT to bank — confirm received &amp; booked</t>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>FIAT to bank</t>
         </is>
       </c>
     </row>
@@ -3507,9 +3596,9 @@
       <c r="D20" s="7" t="n">
         <v>10000</v>
       </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>FIAT to bank — confirm received &amp; booked</t>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>FIAT to bank</t>
         </is>
       </c>
     </row>
@@ -3524,9 +3613,9 @@
       <c r="D21" s="7" t="n">
         <v>50000</v>
       </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>PRE-PERIOD (Aug 2024); no trace on-chain or booked — confirm ever received</t>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>PRE-PERIOD; no trace — confirm received</t>
         </is>
       </c>
     </row>
@@ -3541,9 +3630,9 @@
       </c>
       <c r="C22" s="5" t="n"/>
       <c r="D22" s="5" t="n"/>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>On-chain into Op Hub — NON-INVESTOR receipt (book as other income)</t>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>NON-INVESTOR receipt to Op Hub (other income)</t>
         </is>
       </c>
     </row>
@@ -3558,19 +3647,568 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Arbitrum — FY25 in-period (NEW: was outside the eth+base trace)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Material FY25 expense missing from the locked accounts. The CEH wallet was the team payroll hub on Arbitrum Feb-Sep 2025. 2026 Arbitrum trading (~$29m) is post-period FY26 own infra, excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>A) Group → CEH wallet (payroll funding)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>2025-02-28</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>35900</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>2025-02-28</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>2025-03-27</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>2025-04-30</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>41000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>2025-05-29</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>41000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>2025-06-27</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>41000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>2025-07-30</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>41000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>2025-08-29</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>40999.95</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>2025-09-26</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>41000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>317999.95</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>B) CEH → team / contractor fan-out (distribution of the above)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Payee</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Josh Hardy</t>
+        </is>
+      </c>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>0x2452bebf24353f1ac39b8252f40f8fd7e4be4be2</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>78000</v>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>2025-03-01-&gt;2025-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>0xa9d6ab42f32dc476269db2407715d8c15a36d781</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="n">
+        <v>45980</v>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>2025-03-02-&gt;2025-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Dave Meister (personal)</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>0x1d56a5ed5cbeaa8885bb61c820b7f897da00531c</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="n">
+        <v>36000</v>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>2025-03-01-&gt;2025-05-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>David Atkinson (Rain wallet)</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>0xdf1802c9ab5ed41615cc8db10ee8c1c0ea56dbc7</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="n">
+        <v>27000</v>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>2025-07-01-&gt;2025-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>0xb43b25ec82a030792d4ffac109cdcc353f118d75</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="n">
+        <v>26079</v>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>2025-07-15-&gt;2025-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>0x86aef9beac77fee6f2165e515fce6505f40afc27</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="n">
+        <v>24000</v>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>2025-03-02-&gt;2025-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>0x84d14a8480737c223168b083bcda189ac7783010</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="n">
+        <v>21818.24</v>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>2025-05-01-&gt;2025-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>0x69ecafbac149ab7b0d6af080289542c615e53021</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="n">
+        <v>16480</v>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>2025-02-13-&gt;2025-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>0x9604b25026b3032c06b365df7fc7870c04310600</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="n">
+        <v>14500</v>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>2025-03-02-&gt;2025-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>0xab6306f1fde8fbcdd520ca2b151d45577d46cd31</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="n">
+        <v>14043.65</v>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>2025-03-02-&gt;2025-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>0xc98d0319cc6103ffd8927da690d92bb674b7e9b2</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="n">
+        <v>11482.75</v>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>2025-07-01-&gt;2025-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B30" s="24" t="inlineStr">
+        <is>
+          <t>0x4912428f17380b6ab253ac77479e9bf92ea8dbb0</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="n">
+        <v>10010</v>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>2025-03-03-&gt;2025-05-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>0x228b84155dff69f30fae77a008762087ac8e62b8</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="n">
+        <v>9990</v>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>2025-03-03-&gt;2025-05-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B32" s="24" t="inlineStr">
+        <is>
+          <t>0xd43ca531907f8c8dbb3272cc2ef321cc572e56e3</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="n">
+        <v>5580</v>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>2025-05-01-&gt;2025-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>Team/contractor payee (unidentified)</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>0x9008d19f58aabd9ed0d60971565aa8510560ab41</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="n">
+        <v>1201.11</v>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>2025-07-31-&gt;2025-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="22" t="inlineStr">
+        <is>
+          <t>Total distributed</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="n">
+        <v>342165</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Plus $60k CEH on Ethereum mainnet (Oct-Dec 2025). CEH true group cost ≈ $378k vs $60k previously recorded.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Open items / flags for Count &amp; Tom Fleming</t>
+          <t>Open items / flags</t>
         </is>
       </c>
     </row>
@@ -3602,17 +4240,17 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Six fiat ASAs (~$112k): Hoyland 33k, Vantage 30k, CTRL-H 15k, Spitzform 12.5k, Schoofs 11.75k, Middleton 10k</t>
+          <t>Arbitrum payroll via CEH — $318k in-period (FY25)</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Confirm cash landed in Revolut and booked to 951</t>
+          <t>Book as dev/payroll expense; reconcile CEH to $378k total. Post-gate discovery (gate closed 9 Jun).</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>Tom Fleming</t>
         </is>
       </c>
     </row>
@@ -3622,17 +4260,17 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Mark Heus Dec $100k SAFT</t>
+          <t>2026 Arbitrum trading (~$29m, own ops/MM/bridge)</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Confirm timing: ~$24k on-chain in-period, rest post-period/unfunded</t>
+          <t>FY26 not FY25 — exclude from these accounts; sweep separately for FY26</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>Count / Nick</t>
         </is>
       </c>
     </row>
@@ -3642,12 +4280,12 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>K&amp;Co December tranches</t>
+          <t>Six fiat ASAs (~$112k): Hoyland, Vantage, CTRL-H, Spitzform, Schoofs, Middleton</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Align $100k Nov SAFT + $65k to on-chain legs ($24,700 2 Dec + $65k 23 Dec)</t>
+          <t>Confirm cash landed in Revolut and booked</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -3662,12 +4300,12 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Sean $150k W4 Apr leg</t>
+          <t>Mark Heus Dec $100k SAFT / K&amp;Co Dec tranches</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>On-chain source wallet differs from Xero assumption — confirm source</t>
+          <t>Align timing and legs</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -3682,12 +4320,12 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>ultrahd.eth $3,000 into Op Hub (Nov 2025)</t>
+          <t>Sean $150k W4 Apr leg</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Book as other income / refund, not share premium</t>
+          <t>Confirm on-chain source</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -3702,12 +4340,12 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Derk Griffioen $50k (pre-period Aug 2024)</t>
+          <t>ultrahd.eth $3,000 into Op Hub</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Confirm whether ever received</t>
+          <t>Book as other income, not share premium</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -3742,17 +4380,17 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Sub-threshold dust $15,175</t>
+          <t>Address-poisoning on CEH/Arbitrum wallets</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Immaterial on-chain fees/dust — no action</t>
+          <t>Addresses from invoice/address book only; verify first+last 8 chars</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DA / Dave</t>
         </is>
       </c>
     </row>

</xml_diff>